<commit_message>
planillas intl: py, do y sv; desplegables con etiquetas oficiales desde la hoja de tablas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/private/intl/ec/sueldo-y-liquidacion-2026.xlsx
+++ b/private/intl/ec/sueldo-y-liquidacion-2026.xlsx
@@ -1459,7 +1459,7 @@
       <formula2>1000000000000</formula2>
     </dataValidation>
     <dataValidation type="list" showErrorMessage="1" error="Elige una opción de la lista." sqref="B8">
-      <formula1>"Sin cargas familiares,1 carga familiar,2 cargas familiares,3 cargas familiares,4 cargas familiares,5 o más cargas familiares"</formula1>
+      <formula1>'Tablas oficiales'!$B$4:$B$9</formula1>
     </dataValidation>
     <dataValidation type="list" showErrorMessage="1" error="Elige una opción de la lista." sqref="B9">
       <formula1>"Sí,No"</formula1>
@@ -1750,7 +1750,7 @@
   </mergeCells>
   <dataValidations count="5">
     <dataValidation type="list" showErrorMessage="1" error="Elige una opción de la lista." sqref="B15">
-      <formula1>"Costa y Galápagos,Sierra y Amazonía"</formula1>
+      <formula1>'Tablas oficiales'!$B$28:$B$29</formula1>
     </dataValidation>
     <dataValidation type="date" operator="greaterThan" allowBlank="1" showErrorMessage="1" error="Escribe una fecha como dd/mm/aaaa." sqref="B16:B17">
       <formula1>18264</formula1>
@@ -2138,7 +2138,7 @@
       <formula1>"Despido intempestivo (sin causa),Renuncia con aviso escrito (desahucio),Acuerdo entre las partes,Visto bueno pedido por el empleador"</formula1>
     </dataValidation>
     <dataValidation type="list" showErrorMessage="1" error="Elige una opción de la lista." sqref="B9">
-      <formula1>"Costa y Galápagos,Sierra y Amazonía"</formula1>
+      <formula1>'Tablas oficiales'!$B$28:$B$29</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>